<commit_message>
Add patient list for Cruz Roja La Candelaria with 31 entries and update consolidated records to include 3 new unique names. Update README with link.
</commit_message>
<xml_diff>
--- a/consolidado.xlsx
+++ b/consolidado.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Consolidado" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Consolidado!$A$1:$G$1115</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Consolidado!$A$1:$G$1118</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6040" uniqueCount="2153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6055" uniqueCount="2158">
   <si>
     <t xml:space="preserve">Consolidado — Heridos y pacientes · Terremoto Venezuela (24/06/2026)</t>
   </si>
@@ -6155,6 +6155,15 @@
     <t xml:space="preserve">Chen Boye</t>
   </si>
   <si>
+    <t xml:space="preserve">Eliana Contreras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lista atendidos Cruz Roja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente: Cruz Roja La Candelaria 26JUN26</t>
+  </si>
+  <si>
     <t xml:space="preserve">Franco Antonio</t>
   </si>
   <si>
@@ -6176,6 +6185,9 @@
     <t xml:space="preserve">Fuente: Consolidado UCV 25JUN26 · Tel: 4806707</t>
   </si>
   <si>
+    <t xml:space="preserve">Helena Acevedo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hernández Jackeline</t>
   </si>
   <si>
@@ -6237,6 +6249,9 @@
   </si>
   <si>
     <t xml:space="preserve">Tingy José</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeria Castillo</t>
   </si>
   <si>
     <t xml:space="preserve">Varela Angel</t>
@@ -7204,7 +7219,7 @@
       </c>
       <c r="B14" s="5" t="n">
         <f aca="false">COUNTIF(Consolidado!$A:$A,A14)</f>
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">COUNTIFS(Consolidado!$A:$A,A14,Consolidado!$G:$G,"*Consolidado UCV*")</f>
@@ -7243,7 +7258,7 @@
       </c>
       <c r="B17" s="7" t="n">
         <f aca="false">SUM(B5:B16)</f>
-        <v>1114</v>
+        <v>1117</v>
       </c>
       <c r="C17" s="7" t="n">
         <f aca="false">SUM(C5:C16)</f>
@@ -7301,7 +7316,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1115"/>
+  <dimension ref="A1:G1118"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -27877,24 +27892,22 @@
       </c>
     </row>
     <row r="1040" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1040" s="17" t="s">
+      <c r="A1040" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B1040" s="18" t="s">
+      <c r="B1040" s="11" t="s">
         <v>2043</v>
       </c>
-      <c r="C1040" s="19" t="s">
-        <v>801</v>
-      </c>
-      <c r="D1040" s="20"/>
-      <c r="E1040" s="17" t="s">
+      <c r="C1040" s="12"/>
+      <c r="D1040" s="13"/>
+      <c r="E1040" s="10" t="s">
+        <v>2034</v>
+      </c>
+      <c r="F1040" s="10" t="s">
         <v>2044</v>
       </c>
-      <c r="F1040" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="G1040" s="17" t="s">
-        <v>56</v>
+      <c r="G1040" s="10" t="s">
+        <v>2045</v>
       </c>
     </row>
     <row r="1041" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27902,20 +27915,20 @@
         <v>14</v>
       </c>
       <c r="B1041" s="18" t="s">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="C1041" s="19" t="s">
-        <v>191</v>
+        <v>801</v>
       </c>
       <c r="D1041" s="20"/>
       <c r="E1041" s="17" t="s">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="F1041" s="17" t="s">
         <v>55</v>
       </c>
       <c r="G1041" s="17" t="s">
-        <v>2047</v>
+        <v>56</v>
       </c>
     </row>
     <row r="1042" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27926,17 +27939,17 @@
         <v>2048</v>
       </c>
       <c r="C1042" s="19" t="s">
-        <v>394</v>
+        <v>191</v>
       </c>
       <c r="D1042" s="20"/>
       <c r="E1042" s="17" t="s">
-        <v>2034</v>
+        <v>2049</v>
       </c>
       <c r="F1042" s="17" t="s">
         <v>55</v>
       </c>
       <c r="G1042" s="17" t="s">
-        <v>2049</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="1043" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27944,41 +27957,39 @@
         <v>14</v>
       </c>
       <c r="B1043" s="18" t="s">
-        <v>2050</v>
+        <v>2051</v>
       </c>
       <c r="C1043" s="19" t="s">
-        <v>722</v>
+        <v>394</v>
       </c>
       <c r="D1043" s="20"/>
       <c r="E1043" s="17" t="s">
-        <v>2051</v>
+        <v>2034</v>
       </c>
       <c r="F1043" s="17" t="s">
         <v>55</v>
       </c>
       <c r="G1043" s="17" t="s">
-        <v>56</v>
+        <v>2052</v>
       </c>
     </row>
     <row r="1044" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1044" s="17" t="s">
+      <c r="A1044" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B1044" s="18" t="s">
-        <v>2052</v>
-      </c>
-      <c r="C1044" s="19" t="s">
+      <c r="B1044" s="11" t="s">
         <v>2053</v>
       </c>
-      <c r="D1044" s="20"/>
-      <c r="E1044" s="17" t="s">
+      <c r="C1044" s="12"/>
+      <c r="D1044" s="13"/>
+      <c r="E1044" s="10" t="s">
         <v>2034</v>
       </c>
-      <c r="F1044" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="G1044" s="17" t="s">
-        <v>56</v>
+      <c r="F1044" s="10" t="s">
+        <v>2044</v>
+      </c>
+      <c r="G1044" s="10" t="s">
+        <v>2045</v>
       </c>
     </row>
     <row r="1045" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27989,11 +28000,11 @@
         <v>2054</v>
       </c>
       <c r="C1045" s="19" t="s">
-        <v>73</v>
+        <v>722</v>
       </c>
       <c r="D1045" s="20"/>
       <c r="E1045" s="17" t="s">
-        <v>2034</v>
+        <v>2055</v>
       </c>
       <c r="F1045" s="17" t="s">
         <v>55</v>
@@ -28007,10 +28018,10 @@
         <v>14</v>
       </c>
       <c r="B1046" s="18" t="s">
-        <v>2055</v>
+        <v>2056</v>
       </c>
       <c r="C1046" s="19" t="s">
-        <v>926</v>
+        <v>2057</v>
       </c>
       <c r="D1046" s="20"/>
       <c r="E1046" s="17" t="s">
@@ -28028,10 +28039,10 @@
         <v>14</v>
       </c>
       <c r="B1047" s="18" t="s">
-        <v>2056</v>
+        <v>2058</v>
       </c>
       <c r="C1047" s="19" t="s">
-        <v>368</v>
+        <v>73</v>
       </c>
       <c r="D1047" s="20"/>
       <c r="E1047" s="17" t="s">
@@ -28049,10 +28060,10 @@
         <v>14</v>
       </c>
       <c r="B1048" s="18" t="s">
-        <v>2057</v>
+        <v>2059</v>
       </c>
       <c r="C1048" s="19" t="s">
-        <v>68</v>
+        <v>926</v>
       </c>
       <c r="D1048" s="20"/>
       <c r="E1048" s="17" t="s">
@@ -28070,14 +28081,14 @@
         <v>14</v>
       </c>
       <c r="B1049" s="18" t="s">
-        <v>2058</v>
+        <v>2060</v>
       </c>
       <c r="C1049" s="19" t="s">
-        <v>50</v>
+        <v>368</v>
       </c>
       <c r="D1049" s="20"/>
       <c r="E1049" s="17" t="s">
-        <v>2059</v>
+        <v>2034</v>
       </c>
       <c r="F1049" s="17" t="s">
         <v>55</v>
@@ -28091,10 +28102,10 @@
         <v>14</v>
       </c>
       <c r="B1050" s="18" t="s">
-        <v>2060</v>
+        <v>2061</v>
       </c>
       <c r="C1050" s="19" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="D1050" s="20"/>
       <c r="E1050" s="17" t="s">
@@ -28112,14 +28123,14 @@
         <v>14</v>
       </c>
       <c r="B1051" s="18" t="s">
-        <v>2061</v>
+        <v>2062</v>
       </c>
       <c r="C1051" s="19" t="s">
-        <v>298</v>
+        <v>50</v>
       </c>
       <c r="D1051" s="20"/>
       <c r="E1051" s="17" t="s">
-        <v>2034</v>
+        <v>2063</v>
       </c>
       <c r="F1051" s="17" t="s">
         <v>55</v>
@@ -28133,10 +28144,10 @@
         <v>14</v>
       </c>
       <c r="B1052" s="18" t="s">
-        <v>2062</v>
+        <v>2064</v>
       </c>
       <c r="C1052" s="19" t="s">
-        <v>394</v>
+        <v>41</v>
       </c>
       <c r="D1052" s="20"/>
       <c r="E1052" s="17" t="s">
@@ -28154,20 +28165,20 @@
         <v>14</v>
       </c>
       <c r="B1053" s="18" t="s">
-        <v>2063</v>
+        <v>2065</v>
       </c>
       <c r="C1053" s="19" t="s">
         <v>298</v>
       </c>
       <c r="D1053" s="20"/>
       <c r="E1053" s="17" t="s">
-        <v>33</v>
+        <v>2034</v>
       </c>
       <c r="F1053" s="17" t="s">
         <v>55</v>
       </c>
       <c r="G1053" s="17" t="s">
-        <v>2064</v>
+        <v>56</v>
       </c>
     </row>
     <row r="1054" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28175,14 +28186,14 @@
         <v>14</v>
       </c>
       <c r="B1054" s="18" t="s">
-        <v>2065</v>
+        <v>2066</v>
       </c>
       <c r="C1054" s="19" t="s">
-        <v>298</v>
+        <v>394</v>
       </c>
       <c r="D1054" s="20"/>
       <c r="E1054" s="17" t="s">
-        <v>2066</v>
+        <v>2034</v>
       </c>
       <c r="F1054" s="17" t="s">
         <v>55</v>
@@ -28199,17 +28210,17 @@
         <v>2067</v>
       </c>
       <c r="C1055" s="19" t="s">
-        <v>251</v>
+        <v>298</v>
       </c>
       <c r="D1055" s="20"/>
       <c r="E1055" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1055" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1055" s="17" t="s">
         <v>2068</v>
-      </c>
-      <c r="F1055" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="G1055" s="17" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="1056" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28220,11 +28231,11 @@
         <v>2069</v>
       </c>
       <c r="C1056" s="19" t="s">
-        <v>287</v>
+        <v>298</v>
       </c>
       <c r="D1056" s="20"/>
       <c r="E1056" s="17" t="s">
-        <v>2068</v>
+        <v>2070</v>
       </c>
       <c r="F1056" s="17" t="s">
         <v>55</v>
@@ -28238,14 +28249,14 @@
         <v>14</v>
       </c>
       <c r="B1057" s="18" t="s">
-        <v>2070</v>
+        <v>2071</v>
       </c>
       <c r="C1057" s="19" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="D1057" s="20"/>
       <c r="E1057" s="17" t="s">
-        <v>2034</v>
+        <v>2072</v>
       </c>
       <c r="F1057" s="17" t="s">
         <v>55</v>
@@ -28259,14 +28270,14 @@
         <v>14</v>
       </c>
       <c r="B1058" s="18" t="s">
-        <v>2071</v>
+        <v>2073</v>
       </c>
       <c r="C1058" s="19" t="s">
-        <v>68</v>
+        <v>287</v>
       </c>
       <c r="D1058" s="20"/>
       <c r="E1058" s="17" t="s">
-        <v>2038</v>
+        <v>2072</v>
       </c>
       <c r="F1058" s="17" t="s">
         <v>55</v>
@@ -28280,13 +28291,15 @@
         <v>14</v>
       </c>
       <c r="B1059" s="18" t="s">
-        <v>2072</v>
+        <v>2074</v>
       </c>
       <c r="C1059" s="19" t="s">
-        <v>287</v>
+        <v>260</v>
       </c>
       <c r="D1059" s="20"/>
-      <c r="E1059" s="17"/>
+      <c r="E1059" s="17" t="s">
+        <v>2034</v>
+      </c>
       <c r="F1059" s="17" t="s">
         <v>55</v>
       </c>
@@ -28295,43 +28308,37 @@
       </c>
     </row>
     <row r="1060" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1060" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1060" s="18" t="s">
-        <v>2073</v>
-      </c>
-      <c r="C1060" s="19" t="s">
-        <v>740</v>
-      </c>
-      <c r="D1060" s="20" t="s">
-        <v>2074</v>
-      </c>
-      <c r="E1060" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="F1060" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="G1060" s="17" t="s">
-        <v>56</v>
+      <c r="A1060" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1060" s="11" t="s">
+        <v>2075</v>
+      </c>
+      <c r="C1060" s="12"/>
+      <c r="D1060" s="13"/>
+      <c r="E1060" s="10" t="s">
+        <v>2034</v>
+      </c>
+      <c r="F1060" s="10" t="s">
+        <v>2044</v>
+      </c>
+      <c r="G1060" s="10" t="s">
+        <v>2045</v>
       </c>
     </row>
     <row r="1061" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1061" s="17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1061" s="18" t="s">
-        <v>2075</v>
+        <v>2076</v>
       </c>
       <c r="C1061" s="19" t="s">
-        <v>332</v>
-      </c>
-      <c r="D1061" s="20" t="s">
-        <v>2076</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="D1061" s="20"/>
       <c r="E1061" s="17" t="s">
-        <v>33</v>
+        <v>2038</v>
       </c>
       <c r="F1061" s="17" t="s">
         <v>55</v>
@@ -28342,20 +28349,16 @@
     </row>
     <row r="1062" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1062" s="17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1062" s="18" t="s">
         <v>2077</v>
       </c>
       <c r="C1062" s="19" t="s">
-        <v>1045</v>
-      </c>
-      <c r="D1062" s="20" t="s">
-        <v>2078</v>
-      </c>
-      <c r="E1062" s="17" t="s">
-        <v>33</v>
-      </c>
+        <v>287</v>
+      </c>
+      <c r="D1062" s="20"/>
+      <c r="E1062" s="17"/>
       <c r="F1062" s="17" t="s">
         <v>55</v>
       </c>
@@ -28368,13 +28371,13 @@
         <v>15</v>
       </c>
       <c r="B1063" s="18" t="s">
-        <v>2079</v>
+        <v>2078</v>
       </c>
       <c r="C1063" s="19" t="s">
         <v>740</v>
       </c>
       <c r="D1063" s="20" t="s">
-        <v>2080</v>
+        <v>2079</v>
       </c>
       <c r="E1063" s="17" t="s">
         <v>33</v>
@@ -28391,16 +28394,16 @@
         <v>15</v>
       </c>
       <c r="B1064" s="18" t="s">
+        <v>2080</v>
+      </c>
+      <c r="C1064" s="19" t="s">
+        <v>332</v>
+      </c>
+      <c r="D1064" s="20" t="s">
         <v>2081</v>
       </c>
-      <c r="C1064" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="D1064" s="20" t="s">
-        <v>2082</v>
-      </c>
       <c r="E1064" s="17" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="F1064" s="17" t="s">
         <v>55</v>
@@ -28414,13 +28417,13 @@
         <v>15</v>
       </c>
       <c r="B1065" s="18" t="s">
+        <v>2082</v>
+      </c>
+      <c r="C1065" s="19" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D1065" s="20" t="s">
         <v>2083</v>
-      </c>
-      <c r="C1065" s="19" t="s">
-        <v>771</v>
-      </c>
-      <c r="D1065" s="20" t="s">
-        <v>2084</v>
       </c>
       <c r="E1065" s="17" t="s">
         <v>33</v>
@@ -28437,13 +28440,13 @@
         <v>15</v>
       </c>
       <c r="B1066" s="18" t="s">
+        <v>2084</v>
+      </c>
+      <c r="C1066" s="19" t="s">
+        <v>740</v>
+      </c>
+      <c r="D1066" s="20" t="s">
         <v>2085</v>
-      </c>
-      <c r="C1066" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="D1066" s="20" t="s">
-        <v>2086</v>
       </c>
       <c r="E1066" s="17" t="s">
         <v>33</v>
@@ -28460,16 +28463,16 @@
         <v>15</v>
       </c>
       <c r="B1067" s="18" t="s">
+        <v>2086</v>
+      </c>
+      <c r="C1067" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1067" s="20" t="s">
         <v>2087</v>
       </c>
-      <c r="C1067" s="19" t="s">
-        <v>2088</v>
-      </c>
-      <c r="D1067" s="20" t="s">
-        <v>2089</v>
-      </c>
       <c r="E1067" s="17" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="F1067" s="17" t="s">
         <v>55</v>
@@ -28483,13 +28486,13 @@
         <v>15</v>
       </c>
       <c r="B1068" s="18" t="s">
-        <v>2090</v>
+        <v>2088</v>
       </c>
       <c r="C1068" s="19" t="s">
-        <v>167</v>
+        <v>771</v>
       </c>
       <c r="D1068" s="20" t="s">
-        <v>2091</v>
+        <v>2089</v>
       </c>
       <c r="E1068" s="17" t="s">
         <v>33</v>
@@ -28506,16 +28509,16 @@
         <v>15</v>
       </c>
       <c r="B1069" s="18" t="s">
-        <v>2092</v>
+        <v>2090</v>
       </c>
       <c r="C1069" s="19" t="s">
-        <v>160</v>
+        <v>307</v>
       </c>
       <c r="D1069" s="20" t="s">
-        <v>2093</v>
+        <v>2091</v>
       </c>
       <c r="E1069" s="17" t="s">
-        <v>2094</v>
+        <v>33</v>
       </c>
       <c r="F1069" s="17" t="s">
         <v>55</v>
@@ -28529,16 +28532,16 @@
         <v>15</v>
       </c>
       <c r="B1070" s="18" t="s">
-        <v>2095</v>
+        <v>2092</v>
       </c>
       <c r="C1070" s="19" t="s">
-        <v>58</v>
+        <v>2093</v>
       </c>
       <c r="D1070" s="20" t="s">
-        <v>2096</v>
+        <v>2094</v>
       </c>
       <c r="E1070" s="17" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="F1070" s="17" t="s">
         <v>55</v>
@@ -28552,13 +28555,13 @@
         <v>15</v>
       </c>
       <c r="B1071" s="18" t="s">
-        <v>2097</v>
+        <v>2095</v>
       </c>
       <c r="C1071" s="19" t="s">
-        <v>817</v>
+        <v>167</v>
       </c>
       <c r="D1071" s="20" t="s">
-        <v>2098</v>
+        <v>2096</v>
       </c>
       <c r="E1071" s="17" t="s">
         <v>33</v>
@@ -28575,16 +28578,16 @@
         <v>15</v>
       </c>
       <c r="B1072" s="18" t="s">
-        <v>1596</v>
+        <v>2097</v>
       </c>
       <c r="C1072" s="19" t="s">
-        <v>332</v>
+        <v>160</v>
       </c>
       <c r="D1072" s="20" t="s">
+        <v>2098</v>
+      </c>
+      <c r="E1072" s="17" t="s">
         <v>2099</v>
-      </c>
-      <c r="E1072" s="17" t="s">
-        <v>33</v>
       </c>
       <c r="F1072" s="17" t="s">
         <v>55</v>
@@ -28601,13 +28604,13 @@
         <v>2100</v>
       </c>
       <c r="C1073" s="19" t="s">
-        <v>135</v>
+        <v>58</v>
       </c>
       <c r="D1073" s="20" t="s">
         <v>2101</v>
       </c>
       <c r="E1073" s="17" t="s">
-        <v>2102</v>
+        <v>33</v>
       </c>
       <c r="F1073" s="17" t="s">
         <v>55</v>
@@ -28621,13 +28624,13 @@
         <v>15</v>
       </c>
       <c r="B1074" s="18" t="s">
+        <v>2102</v>
+      </c>
+      <c r="C1074" s="19" t="s">
+        <v>817</v>
+      </c>
+      <c r="D1074" s="20" t="s">
         <v>2103</v>
-      </c>
-      <c r="C1074" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="D1074" s="20" t="s">
-        <v>2104</v>
       </c>
       <c r="E1074" s="17" t="s">
         <v>33</v>
@@ -28644,13 +28647,13 @@
         <v>15</v>
       </c>
       <c r="B1075" s="18" t="s">
-        <v>2105</v>
+        <v>1596</v>
       </c>
       <c r="C1075" s="19" t="s">
-        <v>1264</v>
+        <v>332</v>
       </c>
       <c r="D1075" s="20" t="s">
-        <v>2106</v>
+        <v>2104</v>
       </c>
       <c r="E1075" s="17" t="s">
         <v>33</v>
@@ -28667,16 +28670,16 @@
         <v>15</v>
       </c>
       <c r="B1076" s="18" t="s">
+        <v>2105</v>
+      </c>
+      <c r="C1076" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1076" s="20" t="s">
+        <v>2106</v>
+      </c>
+      <c r="E1076" s="17" t="s">
         <v>2107</v>
-      </c>
-      <c r="C1076" s="19" t="s">
-        <v>1037</v>
-      </c>
-      <c r="D1076" s="20" t="s">
-        <v>2108</v>
-      </c>
-      <c r="E1076" s="17" t="s">
-        <v>2109</v>
       </c>
       <c r="F1076" s="17" t="s">
         <v>55</v>
@@ -28690,13 +28693,13 @@
         <v>15</v>
       </c>
       <c r="B1077" s="18" t="s">
-        <v>2110</v>
+        <v>2108</v>
       </c>
       <c r="C1077" s="19" t="s">
-        <v>740</v>
+        <v>46</v>
       </c>
       <c r="D1077" s="20" t="s">
-        <v>2111</v>
+        <v>2109</v>
       </c>
       <c r="E1077" s="17" t="s">
         <v>33</v>
@@ -28713,13 +28716,13 @@
         <v>15</v>
       </c>
       <c r="B1078" s="18" t="s">
-        <v>2112</v>
+        <v>2110</v>
       </c>
       <c r="C1078" s="19" t="s">
-        <v>981</v>
+        <v>1264</v>
       </c>
       <c r="D1078" s="20" t="s">
-        <v>2113</v>
+        <v>2111</v>
       </c>
       <c r="E1078" s="17" t="s">
         <v>33</v>
@@ -28736,16 +28739,16 @@
         <v>15</v>
       </c>
       <c r="B1079" s="18" t="s">
+        <v>2112</v>
+      </c>
+      <c r="C1079" s="19" t="s">
+        <v>1037</v>
+      </c>
+      <c r="D1079" s="20" t="s">
+        <v>2113</v>
+      </c>
+      <c r="E1079" s="17" t="s">
         <v>2114</v>
-      </c>
-      <c r="C1079" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="D1079" s="20" t="s">
-        <v>2115</v>
-      </c>
-      <c r="E1079" s="17" t="s">
-        <v>33</v>
       </c>
       <c r="F1079" s="17" t="s">
         <v>55</v>
@@ -28759,13 +28762,13 @@
         <v>15</v>
       </c>
       <c r="B1080" s="18" t="s">
+        <v>2115</v>
+      </c>
+      <c r="C1080" s="19" t="s">
+        <v>740</v>
+      </c>
+      <c r="D1080" s="20" t="s">
         <v>2116</v>
-      </c>
-      <c r="C1080" s="19" t="s">
-        <v>731</v>
-      </c>
-      <c r="D1080" s="20" t="s">
-        <v>2117</v>
       </c>
       <c r="E1080" s="17" t="s">
         <v>33</v>
@@ -28782,13 +28785,13 @@
         <v>15</v>
       </c>
       <c r="B1081" s="18" t="s">
+        <v>2117</v>
+      </c>
+      <c r="C1081" s="19" t="s">
+        <v>981</v>
+      </c>
+      <c r="D1081" s="20" t="s">
         <v>2118</v>
-      </c>
-      <c r="C1081" s="19" t="s">
-        <v>251</v>
-      </c>
-      <c r="D1081" s="20" t="s">
-        <v>2119</v>
       </c>
       <c r="E1081" s="17" t="s">
         <v>33</v>
@@ -28802,14 +28805,20 @@
     </row>
     <row r="1082" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1082" s="17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1082" s="18" t="s">
+        <v>2119</v>
+      </c>
+      <c r="C1082" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="D1082" s="20" t="s">
         <v>2120</v>
       </c>
-      <c r="C1082" s="19"/>
-      <c r="D1082" s="20"/>
-      <c r="E1082" s="17"/>
+      <c r="E1082" s="17" t="s">
+        <v>33</v>
+      </c>
       <c r="F1082" s="17" t="s">
         <v>55</v>
       </c>
@@ -28819,14 +28828,20 @@
     </row>
     <row r="1083" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1083" s="17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1083" s="18" t="s">
         <v>2121</v>
       </c>
-      <c r="C1083" s="19"/>
-      <c r="D1083" s="20"/>
-      <c r="E1083" s="17"/>
+      <c r="C1083" s="19" t="s">
+        <v>731</v>
+      </c>
+      <c r="D1083" s="20" t="s">
+        <v>2122</v>
+      </c>
+      <c r="E1083" s="17" t="s">
+        <v>33</v>
+      </c>
       <c r="F1083" s="17" t="s">
         <v>55</v>
       </c>
@@ -28836,14 +28851,20 @@
     </row>
     <row r="1084" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1084" s="17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1084" s="18" t="s">
-        <v>2122</v>
-      </c>
-      <c r="C1084" s="19"/>
-      <c r="D1084" s="20"/>
-      <c r="E1084" s="17"/>
+        <v>2123</v>
+      </c>
+      <c r="C1084" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="D1084" s="20" t="s">
+        <v>2124</v>
+      </c>
+      <c r="E1084" s="17" t="s">
+        <v>33</v>
+      </c>
       <c r="F1084" s="17" t="s">
         <v>55</v>
       </c>
@@ -28856,7 +28877,7 @@
         <v>16</v>
       </c>
       <c r="B1085" s="18" t="s">
-        <v>2123</v>
+        <v>2125</v>
       </c>
       <c r="C1085" s="19"/>
       <c r="D1085" s="20"/>
@@ -28873,7 +28894,7 @@
         <v>16</v>
       </c>
       <c r="B1086" s="18" t="s">
-        <v>2124</v>
+        <v>2126</v>
       </c>
       <c r="C1086" s="19"/>
       <c r="D1086" s="20"/>
@@ -28890,7 +28911,7 @@
         <v>16</v>
       </c>
       <c r="B1087" s="18" t="s">
-        <v>2125</v>
+        <v>2127</v>
       </c>
       <c r="C1087" s="19"/>
       <c r="D1087" s="20"/>
@@ -28907,7 +28928,7 @@
         <v>16</v>
       </c>
       <c r="B1088" s="18" t="s">
-        <v>2126</v>
+        <v>2128</v>
       </c>
       <c r="C1088" s="19"/>
       <c r="D1088" s="20"/>
@@ -28924,7 +28945,7 @@
         <v>16</v>
       </c>
       <c r="B1089" s="18" t="s">
-        <v>2127</v>
+        <v>2129</v>
       </c>
       <c r="C1089" s="19"/>
       <c r="D1089" s="20"/>
@@ -28941,7 +28962,7 @@
         <v>16</v>
       </c>
       <c r="B1090" s="18" t="s">
-        <v>2128</v>
+        <v>2130</v>
       </c>
       <c r="C1090" s="19"/>
       <c r="D1090" s="20"/>
@@ -28958,7 +28979,7 @@
         <v>16</v>
       </c>
       <c r="B1091" s="18" t="s">
-        <v>2129</v>
+        <v>2131</v>
       </c>
       <c r="C1091" s="19"/>
       <c r="D1091" s="20"/>
@@ -28975,7 +28996,7 @@
         <v>16</v>
       </c>
       <c r="B1092" s="18" t="s">
-        <v>2130</v>
+        <v>2132</v>
       </c>
       <c r="C1092" s="19"/>
       <c r="D1092" s="20"/>
@@ -28992,7 +29013,7 @@
         <v>16</v>
       </c>
       <c r="B1093" s="18" t="s">
-        <v>2131</v>
+        <v>2133</v>
       </c>
       <c r="C1093" s="19"/>
       <c r="D1093" s="20"/>
@@ -29009,7 +29030,7 @@
         <v>16</v>
       </c>
       <c r="B1094" s="18" t="s">
-        <v>2132</v>
+        <v>2134</v>
       </c>
       <c r="C1094" s="19"/>
       <c r="D1094" s="20"/>
@@ -29026,7 +29047,7 @@
         <v>16</v>
       </c>
       <c r="B1095" s="18" t="s">
-        <v>2133</v>
+        <v>2135</v>
       </c>
       <c r="C1095" s="19"/>
       <c r="D1095" s="20"/>
@@ -29043,7 +29064,7 @@
         <v>16</v>
       </c>
       <c r="B1096" s="18" t="s">
-        <v>2134</v>
+        <v>2136</v>
       </c>
       <c r="C1096" s="19"/>
       <c r="D1096" s="20"/>
@@ -29060,7 +29081,7 @@
         <v>16</v>
       </c>
       <c r="B1097" s="18" t="s">
-        <v>2135</v>
+        <v>2137</v>
       </c>
       <c r="C1097" s="19"/>
       <c r="D1097" s="20"/>
@@ -29077,7 +29098,7 @@
         <v>16</v>
       </c>
       <c r="B1098" s="18" t="s">
-        <v>2136</v>
+        <v>2138</v>
       </c>
       <c r="C1098" s="19"/>
       <c r="D1098" s="20"/>
@@ -29094,7 +29115,7 @@
         <v>16</v>
       </c>
       <c r="B1099" s="18" t="s">
-        <v>2137</v>
+        <v>2139</v>
       </c>
       <c r="C1099" s="19"/>
       <c r="D1099" s="20"/>
@@ -29111,7 +29132,7 @@
         <v>16</v>
       </c>
       <c r="B1100" s="18" t="s">
-        <v>2138</v>
+        <v>2140</v>
       </c>
       <c r="C1100" s="19"/>
       <c r="D1100" s="20"/>
@@ -29128,7 +29149,7 @@
         <v>16</v>
       </c>
       <c r="B1101" s="18" t="s">
-        <v>2139</v>
+        <v>2141</v>
       </c>
       <c r="C1101" s="19"/>
       <c r="D1101" s="20"/>
@@ -29145,7 +29166,7 @@
         <v>16</v>
       </c>
       <c r="B1102" s="18" t="s">
-        <v>2140</v>
+        <v>2142</v>
       </c>
       <c r="C1102" s="19"/>
       <c r="D1102" s="20"/>
@@ -29162,7 +29183,7 @@
         <v>16</v>
       </c>
       <c r="B1103" s="18" t="s">
-        <v>2141</v>
+        <v>2143</v>
       </c>
       <c r="C1103" s="19"/>
       <c r="D1103" s="20"/>
@@ -29179,7 +29200,7 @@
         <v>16</v>
       </c>
       <c r="B1104" s="18" t="s">
-        <v>2142</v>
+        <v>2144</v>
       </c>
       <c r="C1104" s="19"/>
       <c r="D1104" s="20"/>
@@ -29196,7 +29217,7 @@
         <v>16</v>
       </c>
       <c r="B1105" s="18" t="s">
-        <v>2143</v>
+        <v>2145</v>
       </c>
       <c r="C1105" s="19"/>
       <c r="D1105" s="20"/>
@@ -29213,7 +29234,7 @@
         <v>16</v>
       </c>
       <c r="B1106" s="18" t="s">
-        <v>2144</v>
+        <v>2146</v>
       </c>
       <c r="C1106" s="19"/>
       <c r="D1106" s="20"/>
@@ -29230,7 +29251,7 @@
         <v>16</v>
       </c>
       <c r="B1107" s="18" t="s">
-        <v>2145</v>
+        <v>2147</v>
       </c>
       <c r="C1107" s="19"/>
       <c r="D1107" s="20"/>
@@ -29247,7 +29268,7 @@
         <v>16</v>
       </c>
       <c r="B1108" s="18" t="s">
-        <v>2146</v>
+        <v>2148</v>
       </c>
       <c r="C1108" s="19"/>
       <c r="D1108" s="20"/>
@@ -29264,7 +29285,7 @@
         <v>16</v>
       </c>
       <c r="B1109" s="18" t="s">
-        <v>2147</v>
+        <v>2149</v>
       </c>
       <c r="C1109" s="19"/>
       <c r="D1109" s="20"/>
@@ -29281,7 +29302,7 @@
         <v>16</v>
       </c>
       <c r="B1110" s="18" t="s">
-        <v>2148</v>
+        <v>2150</v>
       </c>
       <c r="C1110" s="19"/>
       <c r="D1110" s="20"/>
@@ -29298,7 +29319,7 @@
         <v>16</v>
       </c>
       <c r="B1111" s="18" t="s">
-        <v>1431</v>
+        <v>2151</v>
       </c>
       <c r="C1111" s="19"/>
       <c r="D1111" s="20"/>
@@ -29315,7 +29336,7 @@
         <v>16</v>
       </c>
       <c r="B1112" s="18" t="s">
-        <v>2149</v>
+        <v>2152</v>
       </c>
       <c r="C1112" s="19"/>
       <c r="D1112" s="20"/>
@@ -29332,7 +29353,7 @@
         <v>16</v>
       </c>
       <c r="B1113" s="18" t="s">
-        <v>2150</v>
+        <v>2153</v>
       </c>
       <c r="C1113" s="19"/>
       <c r="D1113" s="20"/>
@@ -29349,7 +29370,7 @@
         <v>16</v>
       </c>
       <c r="B1114" s="18" t="s">
-        <v>2151</v>
+        <v>1431</v>
       </c>
       <c r="C1114" s="19"/>
       <c r="D1114" s="20"/>
@@ -29366,7 +29387,7 @@
         <v>16</v>
       </c>
       <c r="B1115" s="18" t="s">
-        <v>2152</v>
+        <v>2154</v>
       </c>
       <c r="C1115" s="19"/>
       <c r="D1115" s="20"/>
@@ -29378,8 +29399,59 @@
         <v>56</v>
       </c>
     </row>
+    <row r="1116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1116" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1116" s="18" t="s">
+        <v>2155</v>
+      </c>
+      <c r="C1116" s="19"/>
+      <c r="D1116" s="20"/>
+      <c r="E1116" s="17"/>
+      <c r="F1116" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1116" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1117" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1117" s="18" t="s">
+        <v>2156</v>
+      </c>
+      <c r="C1117" s="19"/>
+      <c r="D1117" s="20"/>
+      <c r="E1117" s="17"/>
+      <c r="F1117" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1117" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1118" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1118" s="18" t="s">
+        <v>2157</v>
+      </c>
+      <c r="C1118" s="19"/>
+      <c r="D1118" s="20"/>
+      <c r="E1118" s="17"/>
+      <c r="F1118" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1118" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1115"/>
+  <autoFilter ref="A1:G1118"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>